<commit_message>
program create issue fix
</commit_message>
<xml_diff>
--- a/dc-uat-checklist-updated.xlsx
+++ b/dc-uat-checklist-updated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\daycare-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AEAC74A-89F9-4C54-81C0-14457124E693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5851DC6-6DF7-4DEC-A303-AF0E4799F91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="573">
   <si>
     <t>Emagine U At Play — UAT Checklist</t>
   </si>
@@ -1802,6 +1802,12 @@
   </si>
   <si>
     <t>Child View Needed</t>
+  </si>
+  <si>
+    <t>authorized for pickup - not showing</t>
+  </si>
+  <si>
+    <t>is_primary=true not marked in parent list</t>
   </si>
 </sst>
 </file>
@@ -2530,11 +2536,11 @@
       </c>
       <c r="D9" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$127,$B9,'UAT Checklist'!$H$2:$H$127,"Not Tested")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E9" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$127,$B9,'UAT Checklist'!$H$2:$H$127,"Pass")</f>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F9" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$127,$B9,'UAT Checklist'!$H$2:$H$127,"Fail")</f>
@@ -2550,7 +2556,7 @@
       </c>
       <c r="I9" s="7">
         <f t="shared" si="0"/>
-        <v>0.375</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.35">
@@ -2596,11 +2602,11 @@
       </c>
       <c r="D11" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$127,$B11,'UAT Checklist'!$H$2:$H$127,"Not Tested")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E11" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$127,$B11,'UAT Checklist'!$H$2:$H$127,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="6">
         <f>COUNTIFS('UAT Checklist'!$B$2:$B$127,$B11,'UAT Checklist'!$H$2:$H$127,"Fail")</f>
@@ -2616,7 +2622,7 @@
       </c>
       <c r="I11" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.35">
@@ -3157,11 +3163,11 @@
       </c>
       <c r="D28" s="8">
         <f t="shared" si="1"/>
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E28" s="8">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F28" s="8">
         <f t="shared" si="1"/>
@@ -3177,7 +3183,7 @@
       </c>
       <c r="I28" s="9">
         <f t="shared" si="0"/>
-        <v>0.15873015873015872</v>
+        <v>0.20634920634920634</v>
       </c>
     </row>
   </sheetData>
@@ -3919,7 +3925,7 @@
         <v>77</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I24" s="11"/>
       <c r="J24" s="10"/>
@@ -3948,7 +3954,7 @@
         <v>77</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I25" s="11"/>
       <c r="J25" s="10"/>
@@ -3977,7 +3983,7 @@
         <v>68</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I26" s="11"/>
       <c r="J26" s="10"/>
@@ -4006,7 +4012,7 @@
         <v>68</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I27" s="11"/>
       <c r="J27" s="10"/>
@@ -4035,7 +4041,7 @@
         <v>77</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I28" s="11"/>
       <c r="J28" s="10"/>
@@ -4124,7 +4130,9 @@
       <c r="H31" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="I31" s="11"/>
+      <c r="I31" s="11" t="s">
+        <v>571</v>
+      </c>
       <c r="J31" s="10"/>
       <c r="K31" s="10"/>
     </row>
@@ -4153,7 +4161,9 @@
       <c r="H32" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="I32" s="11"/>
+      <c r="I32" s="11" t="s">
+        <v>572</v>
+      </c>
       <c r="J32" s="10"/>
       <c r="K32" s="10"/>
     </row>
@@ -4180,7 +4190,7 @@
         <v>77</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I33" s="11"/>
       <c r="J33" s="10"/>

</xml_diff>